<commit_message>
Historial desde el 13/10 leyendo Drive: registro de cada cambio (cada hora), avance semana a semana y tarjetas que no cortan palabras
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/matriz_fen.xlsx
+++ b/datos/matriz_fen.xlsx
@@ -6,12 +6,12 @@
     <sheet state="visible" name="FEN 2026 SENAMHI" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'FEN 2026 SENAMHI'!$A$3:$N$14</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'FEN 2026 SENAMHI'!$A$3:$N$16</definedName>
   </definedNames>
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="DEv8w9uS1nvq0ppttL927aIjEk5eAYo5Hy3mv/7ze4E="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="Y7aebOOaoe7dhenYWx1RA5abF9eSGQ+7AbtmXKPN8kc="/>
     </ext>
   </extLst>
 </workbook>
@@ -28,7 +28,11 @@
         <t xml:space="preserve">======
 ID#AAACISN_8mA
 Sonia Del Carmen Huaman Lozano (OPP-UPM)    (2026-10-07 22:54:19)
-la meta establece 2 informes técnicos, se debe indicar si se emitieron los informes</t>
+la meta establece 2 informes técnicos, se debe indicar si se emitieron los informes
+------
+ID#AAACIZDR8N0
+Julia Y. Acuña Azarte (DHI-SPH)    (2026-10-12 20:44:06)
+2 informe de aforos SPH</t>
       </text>
     </comment>
     <comment authorId="0" ref="I5">
@@ -51,12 +55,28 @@
 verificar la meta, indica 288 imágenes, es lo que se debe reportar, cuantas imágenes ya se han generado?</t>
       </text>
     </comment>
-    <comment authorId="0" ref="I13">
+    <comment authorId="0" ref="I15">
       <text>
         <t xml:space="preserve">======
 ID#AAACISN_8lw
 Sonia Del Carmen Huaman Lozano (OPP-UPM)    (2026-10-07 22:47:41)
 se sugiere modificar a la cantidad de talleres programados, para este caso se han identificado 9</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="J15">
+      <text>
+        <t xml:space="preserve">======
+ID#AAACIZDR8NU
+Yury Wilson Escajadillo Fernández (DMCA-SVC)    (2026-10-12 19:24:54)
+Se esta evaluando continuar Ruta de El Niño en periodo de lluvias, según disponibilidad presupuestaria</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="J11">
+      <text>
+        <t xml:space="preserve">======
+ID#AAACIZDR8NQ
+Yury Wilson Escajadillo Fernández (DMCA-SVC)    (2026-10-12 19:23:40)
+Se esta planenado una actualizacion para mejorar la pagina del monitor con visualizadores del ISPI más locales.</t>
       </text>
     </comment>
     <comment authorId="0" ref="I10">
@@ -70,14 +90,14 @@
   </commentList>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mgjFc4IHIF7NK8DNBPJ+buucPTN3g=="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId1" roundtripDataSignature="AMtx7mgRFYNHtoLUGBgH0sjk4UkaZT3L8A=="/>
     </ext>
   </extLst>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="131">
   <si>
     <t>f</t>
   </si>
@@ -260,7 +280,22 @@
     </r>
   </si>
   <si>
-    <t>está el portal de ares   https://www.senamhi.gob.pe/?p=ares</t>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t xml:space="preserve">está el portal de ares   </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FF1155CC"/>
+        <sz val="8.0"/>
+        <u/>
+      </rPr>
+      <t>https://www.senamhi.gob.pe/?p=ares</t>
+    </r>
   </si>
   <si>
     <t>|</t>
@@ -568,7 +603,7 @@
       </rPr>
       <t xml:space="preserve">1. Se realizaron la implementación de 03 puntos de monitoreo de la calidad del aire en Madre de Dios, 02 puntos en Cusco, 03 en Loreto. Asimismo, se fortaleció 01 punto de monitoreo de calidad del aire en Huánuco.
 2. Se realizó el Boletín N°01 de la Vigilancia de la calidad del aire en la amazonia peruana en el contexto de el niño - agosto 2026
-Actualemte se viene realizando el Boletín N°02 de la Vigilancia de la calidad del aire en la amazonia peruana en el contexto de el niño - setiembre 2026.
+Actualmente se viene realizando el Boletín N°02 de la Vigilancia de la calidad del aire en la amazonia peruana en el contexto de el niño - setiembre 2026.
 </t>
     </r>
     <r>
@@ -599,6 +634,96 @@
       <t>https://drive.google.com/drive/folders/1Kyvo30tQlD-2fS1bOyouvqw6SWT76SbS?usp=drive_link
 2, https://drive.google.com/drive/folders/1ZzH_MxPedvCNJZScg4-x3z9rqMkoW3O8?usp=drive_link</t>
     </r>
+  </si>
+  <si>
+    <t>Evaluar la influencia del Fenómeno El Niño sobre los incendios forestales en la amazonía peruana y su impacto en la calidad del aire.</t>
+  </si>
+  <si>
+    <t>Elaboración de estudio "Influencia del fenómeno El Niño sobre la dinámica de los incendios forestales y su relación con los niveles de contaminación atmosférica por PM2.5, CO y NO2 en los departamentos de Madre de Dios, Cusco y Loreto durante el periodo 2018-2026"</t>
+  </si>
+  <si>
+    <t>Estudio preliminar</t>
+  </si>
+  <si>
+    <t>N° estudios preliminares</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t xml:space="preserve">Avance al 45% durante el periodo programado. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t xml:space="preserve">1. Sistematización de la red de monitoreo de la calidad del aire implementada que considera Madre de Dios, Cusco y Loreto. 
+2. Elaboración del marco conceptual y metodológico del estudio mediante la recopilación de antecedentes nacionales e internacionales.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FFFF0000"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>(reportado 3 de octubre)</t>
+    </r>
+  </si>
+  <si>
+    <t>https://drive.google.com/drive/folders/16A__GAoXmhPrJb8l05JIbvltFaInQ6f_?usp=sharing</t>
+  </si>
+  <si>
+    <t>Facilitar la visualización y consulta de la información ambiental generada por la SVA en el contexto del Fenómeno El Niño</t>
+  </si>
+  <si>
+    <t>Implementación de tablero digital (dashboard) de visualización y consulta de información ambiental atmosférica a nivel nacional en el contexto del Fenómeno El Niño</t>
+  </si>
+  <si>
+    <t>Tablero digital (dashboard)</t>
+  </si>
+  <si>
+    <t>N° de tableros digitales (dashboard)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t xml:space="preserve">Avance al 30% durante el periodo programado. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color theme="1"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t xml:space="preserve">1. Elaboración del diseño de la estructura del tablero digital en general y para las secciones de calidad de aire, atmósfera global en el Observatorio de Vigilancia Atmosférica Marcapomacoha y monitoreo de radiación ultravioleta.
+2. Actualmente se viene realizando la implementación la sección de calidad de aire en las ciudades de Lima, Iquitos, Huánuco, Cusco y Madre de Dios.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color rgb="FFFF0000"/>
+        <sz val="8.0"/>
+      </rPr>
+      <t>(reportado 3 de octubre)</t>
+    </r>
+  </si>
+  <si>
+    <t>https://drive.google.com/drive/folders/1VBxnyGntnLLRkMpUkyRpeFTKSkc2NO83?usp=sharing</t>
   </si>
   <si>
     <t>Vigilancia Climatica para la gestión del riesgo de desastres en el marco del FEN.</t>
@@ -684,10 +809,69 @@
     <t>90% de avance</t>
   </si>
   <si>
-    <t>Em proceso</t>
+    <t>En proceso</t>
   </si>
   <si>
     <t>Avance de 90% del modelo calibrado y validado. En proceso construcción del visor del modelo de inundación</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/drive/folders/1Q1gmpfAz0xKD5FIW89D_X6mlqz9JoFGQ?usp=sharing</t>
+  </si>
+  <si>
+    <t>Fortalecer el monitoreo y pronóstico hidrológico con fines de Alerta temprana  a nivel nacional</t>
+  </si>
+  <si>
+    <t>Utilizar las herramientas de sensoramiento remoto para la evaluación operacional de la humedad del suelo</t>
+  </si>
+  <si>
+    <t>Producto operacional de estimación de la humedad del suelo a través de sensoramiento remoto</t>
+  </si>
+  <si>
+    <t>Visor de humedad del suelo</t>
+  </si>
+  <si>
+    <t>Avance de 90% del modelo calibrado y validado. En proceso construcción del visor del modelo de humedad del suelo</t>
+  </si>
+  <si>
+    <t>Fortalecer el monitoreo y pronóstico hidrológico de ríos amazónicos en base a niveles de agua</t>
+  </si>
+  <si>
+    <t>Utilizar las herramientas de la inteligencia artificial aplicado al modelamiento y pronóstico del nivel de agua de ríos amazónicos</t>
+  </si>
+  <si>
+    <t>Producto operacional de pronóstico diario del nivel de agua de ríos amazónicos</t>
+  </si>
+  <si>
+    <t>Visor AMARU del pronóstico hidrológico diario</t>
+  </si>
+  <si>
+    <t>80% de avance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avance de 80% del modelo calibrado y validado. </t>
+  </si>
+  <si>
+    <t>Fortalecer el monitoreo y análisis de las condiciones atmosféricas mediante la integración y disponibilidad de información de radiosondeo meteorológico en el Observatorio SENAMHI.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implementación y migración del Módulo de Radiosondeo Meteorológico al Sistema Observatorio Nacional de Tiempo, Agua y Clima del Perú del SENAMHI.
+</t>
+  </si>
+  <si>
+    <t>Módulo web de radiosondeo meteorológico implementado e integrado al Observatorio SENAMHI.
+Comprende los puntos de lanzamiento: Lima, Trujillo, Junín, Iquitos, Arequipa y Puno.</t>
+  </si>
+  <si>
+    <t>Número de radiosondajes por día</t>
+  </si>
+  <si>
+    <t>6 radiosondajes por día</t>
+  </si>
+  <si>
+    <t>Se culminó satisfactoriamente la migración e integración del Módulo de Radiosondeo Meteorológico al Observatorio SENAMHI, modernizando su arquitectura tecnológica y centralizando la información en la infraestructura institucional. Se verificó el correcto funcionamiento de los procesos de ingesta, cálculo e interpretación de perfiles atmosféricos, así como la integridad de los datos históricos migrados. La implementación cuenta con el Acta de Conformidad N.° 008-2026-OTI, suscrita el 29 de septiembre de 2026.</t>
+  </si>
+  <si>
+    <t>https://observatorio.senamhi.gob.pe/investigadores/tiempo/radiosondeo</t>
   </si>
 </sst>
 </file>
@@ -849,7 +1033,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -890,6 +1074,9 @@
     <xf borderId="5" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="5" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -908,9 +1095,6 @@
     <xf borderId="5" fillId="5" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="5" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -925,6 +1109,9 @@
     </xf>
     <xf borderId="5" fillId="0" fontId="8" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="5" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1267,12 +1454,12 @@
       <c r="M4" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="N4" s="15" t="s">
+      <c r="N4" s="16" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="5" ht="87.75" customHeight="1">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="17" t="s">
         <v>24</v>
       </c>
       <c r="B5" s="15">
@@ -1296,11 +1483,11 @@
       <c r="H5" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="I5" s="17">
+      <c r="I5" s="18">
         <v>13.0</v>
       </c>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17">
+      <c r="J5" s="18"/>
+      <c r="K5" s="18">
         <v>13.0</v>
       </c>
       <c r="L5" s="14" t="s">
@@ -1319,33 +1506,33 @@
       <c r="C6" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="G6" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="H6" s="18" t="s">
+      <c r="H6" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="I6" s="20" t="s">
+      <c r="I6" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="J6" s="21"/>
-      <c r="K6" s="21"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
       <c r="L6" s="14" t="s">
         <v>21</v>
       </c>
       <c r="M6" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="N6" s="22" t="s">
+      <c r="N6" s="16" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1375,14 +1562,14 @@
       <c r="I7" s="12">
         <v>1.0</v>
       </c>
-      <c r="J7" s="17"/>
-      <c r="K7" s="17">
+      <c r="J7" s="18"/>
+      <c r="K7" s="18">
         <v>1.0</v>
       </c>
       <c r="L7" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="M7" s="22" t="s">
+      <c r="M7" s="16" t="s">
         <v>46</v>
       </c>
       <c r="N7" s="23"/>
@@ -1419,7 +1606,7 @@
       <c r="M8" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="N8" s="22" t="s">
+      <c r="N8" s="16" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1457,11 +1644,11 @@
       <c r="M9" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="N9" s="22" t="s">
+      <c r="N9" s="16" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="10" ht="54.0" customHeight="1">
+    <row r="10" ht="54.0" hidden="1" customHeight="1">
       <c r="A10" s="2"/>
       <c r="B10" s="9">
         <v>7.0</v>
@@ -1484,7 +1671,7 @@
       <c r="H10" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="I10" s="17">
+      <c r="I10" s="18">
         <v>10.0</v>
       </c>
       <c r="J10" s="12"/>
@@ -1535,7 +1722,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="12" ht="73.5" customHeight="1">
+    <row r="12" ht="84.0" customHeight="1">
       <c r="A12" s="2"/>
       <c r="B12" s="9">
         <v>9.0</v>
@@ -1561,8 +1748,8 @@
       <c r="I12" s="12">
         <v>3.0</v>
       </c>
-      <c r="J12" s="17"/>
-      <c r="K12" s="17">
+      <c r="J12" s="18"/>
+      <c r="K12" s="18">
         <v>1.0</v>
       </c>
       <c r="L12" s="15" t="s">
@@ -1571,34 +1758,34 @@
       <c r="M12" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="N12" s="22" t="s">
+      <c r="N12" s="16" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="13" ht="71.25" customHeight="1">
       <c r="A13" s="2"/>
-      <c r="B13" s="9">
+      <c r="B13" s="15">
         <v>10.0</v>
       </c>
       <c r="C13" s="10" t="s">
         <v>32</v>
       </c>
       <c r="D13" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="F13" s="27" t="s">
         <v>80</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="G13" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="G13" s="10" t="s">
+      <c r="H13" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="H13" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="I13" s="12">
+      <c r="I13" s="18">
         <v>1.0</v>
       </c>
       <c r="J13" s="12"/>
@@ -1607,36 +1794,36 @@
         <v>55</v>
       </c>
       <c r="M13" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="N13" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="N13" s="25" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="14" ht="54.0" customHeight="1">
+    </row>
+    <row r="14" ht="71.25" customHeight="1">
       <c r="A14" s="2"/>
-      <c r="B14" s="9">
+      <c r="B14" s="15">
         <v>11.0</v>
       </c>
       <c r="C14" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="18" t="s">
+      <c r="D14" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="E14" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="F14" s="27" t="s">
         <v>86</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="G14" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="F14" s="11" t="s">
+      <c r="H14" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="G14" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="H14" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="I14" s="12">
+      <c r="I14" s="18">
         <v>1.0</v>
       </c>
       <c r="J14" s="12"/>
@@ -1645,167 +1832,279 @@
         <v>55</v>
       </c>
       <c r="M14" s="15" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="N14" s="25" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="15" ht="54.0" customHeight="1">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" ht="71.25" customHeight="1">
       <c r="A15" s="2"/>
       <c r="B15" s="9">
         <v>12.0</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="E15" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="F15" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="F15" s="27" t="s">
+      <c r="G15" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="G15" s="26" t="s">
+      <c r="H15" s="10" t="s">
         <v>95</v>
-      </c>
-      <c r="H15" s="26" t="s">
-        <v>96</v>
       </c>
       <c r="I15" s="12">
         <v>1.0</v>
       </c>
-      <c r="J15" s="13">
-        <v>1.0</v>
-      </c>
-      <c r="K15" s="13" t="s">
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="M15" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="N15" s="25" t="s">
         <v>97</v>
       </c>
-      <c r="L15" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="M15" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="N15" s="15"/>
     </row>
     <row r="16" ht="54.0" customHeight="1">
       <c r="A16" s="2"/>
-      <c r="B16" s="9">
+      <c r="B16" s="15">
         <v>13.0</v>
       </c>
-      <c r="C16" s="10"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="12"/>
+      <c r="C16" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D16" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="I16" s="12">
+        <v>1.0</v>
+      </c>
       <c r="J16" s="12"/>
       <c r="K16" s="12"/>
-      <c r="L16" s="9"/>
-      <c r="M16" s="9"/>
-      <c r="N16" s="9"/>
+      <c r="L16" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="M16" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="N16" s="25" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="17" ht="54.0" customHeight="1">
       <c r="A17" s="2"/>
-      <c r="B17" s="9">
+      <c r="B17" s="15">
         <v>14.0</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="12"/>
-      <c r="J17" s="12"/>
-      <c r="K17" s="12"/>
-      <c r="L17" s="9"/>
-      <c r="M17" s="9"/>
-      <c r="N17" s="9"/>
+      <c r="C17" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E17" s="26" t="s">
+        <v>105</v>
+      </c>
+      <c r="F17" s="27" t="s">
+        <v>106</v>
+      </c>
+      <c r="G17" s="26" t="s">
+        <v>107</v>
+      </c>
+      <c r="H17" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="I17" s="12">
+        <v>1.0</v>
+      </c>
+      <c r="J17" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="K17" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="L17" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="M17" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="N17" s="25" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="18" ht="54.0" customHeight="1">
       <c r="A18" s="2"/>
       <c r="B18" s="9">
         <v>15.0</v>
       </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12"/>
-      <c r="L18" s="9"/>
-      <c r="M18" s="9"/>
-      <c r="N18" s="9"/>
+      <c r="C18" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18" s="26" t="s">
+        <v>113</v>
+      </c>
+      <c r="F18" s="27" t="s">
+        <v>114</v>
+      </c>
+      <c r="G18" s="26" t="s">
+        <v>115</v>
+      </c>
+      <c r="H18" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="I18" s="12">
+        <v>1.0</v>
+      </c>
+      <c r="J18" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="K18" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="L18" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="M18" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="N18" s="25" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="19" ht="54.0" customHeight="1">
       <c r="A19" s="2"/>
-      <c r="B19" s="9">
+      <c r="B19" s="15">
         <v>16.0</v>
       </c>
-      <c r="C19" s="10"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
-      <c r="K19" s="12"/>
-      <c r="L19" s="9"/>
-      <c r="M19" s="9"/>
-      <c r="N19" s="9"/>
+      <c r="C19" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E19" s="26" t="s">
+        <v>118</v>
+      </c>
+      <c r="F19" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="G19" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="H19" s="26" t="s">
+        <v>121</v>
+      </c>
+      <c r="I19" s="12">
+        <v>1.0</v>
+      </c>
+      <c r="J19" s="13">
+        <v>1.0</v>
+      </c>
+      <c r="K19" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="L19" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="M19" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="N19" s="16" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="20" ht="54.0" customHeight="1">
       <c r="A20" s="2"/>
-      <c r="B20" s="9">
+      <c r="B20" s="15">
         <v>17.0</v>
       </c>
-      <c r="C20" s="10"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="12"/>
+      <c r="C20" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="E20" s="26" t="s">
+        <v>124</v>
+      </c>
+      <c r="F20" s="27" t="s">
+        <v>125</v>
+      </c>
+      <c r="G20" s="26" t="s">
+        <v>126</v>
+      </c>
+      <c r="H20" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="I20" s="18" t="s">
+        <v>128</v>
+      </c>
       <c r="J20" s="12"/>
-      <c r="K20" s="12"/>
-      <c r="L20" s="9"/>
-      <c r="M20" s="9"/>
-      <c r="N20" s="9"/>
+      <c r="K20" s="28">
+        <v>1.0</v>
+      </c>
+      <c r="L20" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="M20" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="N20" s="16" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="21" ht="54.0" customHeight="1">
       <c r="A21" s="2"/>
-      <c r="B21" s="9">
-        <v>18.0</v>
+      <c r="B21" s="15">
+        <v>17.0</v>
       </c>
       <c r="C21" s="10"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="12"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="26"/>
+      <c r="I21" s="18"/>
       <c r="J21" s="12"/>
-      <c r="K21" s="12"/>
-      <c r="L21" s="9"/>
-      <c r="M21" s="9"/>
-      <c r="N21" s="9"/>
+      <c r="K21" s="28"/>
+      <c r="L21" s="15"/>
+      <c r="M21" s="15"/>
+      <c r="N21" s="23"/>
     </row>
     <row r="22" ht="54.0" customHeight="1">
       <c r="A22" s="2"/>
       <c r="B22" s="9">
-        <v>19.0</v>
+        <v>18.0</v>
       </c>
       <c r="C22" s="10"/>
-      <c r="D22" s="18"/>
+      <c r="D22" s="19"/>
       <c r="E22" s="10"/>
       <c r="F22" s="11"/>
       <c r="G22" s="10"/>
@@ -1817,85 +2116,95 @@
       <c r="M22" s="9"/>
       <c r="N22" s="9"/>
     </row>
-    <row r="23" ht="15.75" customHeight="1">
+    <row r="23" ht="54.0" customHeight="1">
       <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
-      <c r="M23" s="2"/>
-      <c r="N23" s="2"/>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
+      <c r="B23" s="15">
+        <v>19.0</v>
+      </c>
+      <c r="C23" s="10"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="12"/>
+      <c r="L23" s="9"/>
+      <c r="M23" s="9"/>
+      <c r="N23" s="9"/>
+    </row>
+    <row r="24" ht="54.0" customHeight="1">
       <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
-      <c r="N24" s="2"/>
-    </row>
-    <row r="25" ht="15.75" customHeight="1">
+      <c r="B24" s="15">
+        <v>20.0</v>
+      </c>
+      <c r="C24" s="10"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="12"/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="12"/>
+      <c r="L24" s="9"/>
+      <c r="M24" s="9"/>
+      <c r="N24" s="9"/>
+    </row>
+    <row r="25" ht="54.0" customHeight="1">
       <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
-      <c r="N25" s="2"/>
-    </row>
-    <row r="26" ht="15.75" customHeight="1">
+      <c r="B25" s="9">
+        <v>21.0</v>
+      </c>
+      <c r="C25" s="10"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="12"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="12"/>
+      <c r="L25" s="9"/>
+      <c r="M25" s="9"/>
+      <c r="N25" s="9"/>
+    </row>
+    <row r="26" ht="54.0" customHeight="1">
       <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
-      <c r="L26" s="2"/>
-      <c r="M26" s="2"/>
-      <c r="N26" s="2"/>
-    </row>
-    <row r="27" ht="15.75" customHeight="1">
+      <c r="B26" s="15">
+        <v>22.0</v>
+      </c>
+      <c r="C26" s="10"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="12"/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="12"/>
+      <c r="L26" s="9"/>
+      <c r="M26" s="9"/>
+      <c r="N26" s="9"/>
+    </row>
+    <row r="27" ht="54.0" customHeight="1">
       <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-      <c r="J27" s="2"/>
-      <c r="K27" s="2"/>
-      <c r="L27" s="2"/>
-      <c r="M27" s="2"/>
-      <c r="N27" s="2"/>
+      <c r="B27" s="15">
+        <v>23.0</v>
+      </c>
+      <c r="C27" s="10"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="11"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="12"/>
+      <c r="J27" s="12"/>
+      <c r="K27" s="12"/>
+      <c r="L27" s="9"/>
+      <c r="M27" s="9"/>
+      <c r="N27" s="9"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="2"/>
@@ -16761,8 +17070,96 @@
       <c r="M956" s="2"/>
       <c r="N956" s="2"/>
     </row>
+    <row r="957" ht="15.75" customHeight="1">
+      <c r="A957" s="2"/>
+      <c r="B957" s="2"/>
+      <c r="C957" s="2"/>
+      <c r="D957" s="2"/>
+      <c r="E957" s="2"/>
+      <c r="F957" s="2"/>
+      <c r="G957" s="2"/>
+      <c r="H957" s="2"/>
+      <c r="I957" s="2"/>
+      <c r="J957" s="2"/>
+      <c r="K957" s="2"/>
+      <c r="L957" s="2"/>
+      <c r="M957" s="2"/>
+      <c r="N957" s="2"/>
+    </row>
+    <row r="958" ht="15.75" customHeight="1">
+      <c r="A958" s="2"/>
+      <c r="B958" s="2"/>
+      <c r="C958" s="2"/>
+      <c r="D958" s="2"/>
+      <c r="E958" s="2"/>
+      <c r="F958" s="2"/>
+      <c r="G958" s="2"/>
+      <c r="H958" s="2"/>
+      <c r="I958" s="2"/>
+      <c r="J958" s="2"/>
+      <c r="K958" s="2"/>
+      <c r="L958" s="2"/>
+      <c r="M958" s="2"/>
+      <c r="N958" s="2"/>
+    </row>
+    <row r="959" ht="15.75" customHeight="1">
+      <c r="A959" s="2"/>
+      <c r="B959" s="2"/>
+      <c r="C959" s="2"/>
+      <c r="D959" s="2"/>
+      <c r="E959" s="2"/>
+      <c r="F959" s="2"/>
+      <c r="G959" s="2"/>
+      <c r="H959" s="2"/>
+      <c r="I959" s="2"/>
+      <c r="J959" s="2"/>
+      <c r="K959" s="2"/>
+      <c r="L959" s="2"/>
+      <c r="M959" s="2"/>
+      <c r="N959" s="2"/>
+    </row>
+    <row r="960" ht="15.75" customHeight="1">
+      <c r="A960" s="2"/>
+      <c r="B960" s="2"/>
+      <c r="C960" s="2"/>
+      <c r="D960" s="2"/>
+      <c r="E960" s="2"/>
+      <c r="F960" s="2"/>
+      <c r="G960" s="2"/>
+      <c r="H960" s="2"/>
+      <c r="I960" s="2"/>
+      <c r="J960" s="2"/>
+      <c r="K960" s="2"/>
+      <c r="L960" s="2"/>
+      <c r="M960" s="2"/>
+      <c r="N960" s="2"/>
+    </row>
+    <row r="961" ht="15.75" customHeight="1">
+      <c r="A961" s="2"/>
+      <c r="B961" s="2"/>
+      <c r="C961" s="2"/>
+      <c r="D961" s="2"/>
+      <c r="E961" s="2"/>
+      <c r="F961" s="2"/>
+      <c r="G961" s="2"/>
+      <c r="H961" s="2"/>
+      <c r="I961" s="2"/>
+      <c r="J961" s="2"/>
+      <c r="K961" s="2"/>
+      <c r="L961" s="2"/>
+      <c r="M961" s="2"/>
+      <c r="N961" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="$A$3:$N$14"/>
+  <autoFilter ref="$A$3:$N$16">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Dirección de Meteorología, Clima y Ambiente Atmosférico"/>
+        <filter val="Dirección de Servicios, Cambio Climático y Agrometeorología"/>
+        <filter val="Dirección de Hidrología"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="B2:M2"/>
   </mergeCells>
@@ -16772,19 +17169,26 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId2" ref="N6"/>
-    <hyperlink r:id="rId3" ref="M7"/>
-    <hyperlink r:id="rId4" ref="N8"/>
-    <hyperlink r:id="rId5" ref="N9"/>
-    <hyperlink r:id="rId6" ref="N11"/>
-    <hyperlink r:id="rId7" ref="N12"/>
-    <hyperlink r:id="rId8" ref="N13"/>
-    <hyperlink r:id="rId9" ref="N14"/>
+    <hyperlink r:id="rId2" ref="N4"/>
+    <hyperlink r:id="rId3" ref="N6"/>
+    <hyperlink r:id="rId4" ref="M7"/>
+    <hyperlink r:id="rId5" ref="N8"/>
+    <hyperlink r:id="rId6" ref="N9"/>
+    <hyperlink r:id="rId7" ref="N11"/>
+    <hyperlink r:id="rId8" ref="N12"/>
+    <hyperlink r:id="rId9" ref="N13"/>
+    <hyperlink r:id="rId10" ref="N14"/>
+    <hyperlink r:id="rId11" ref="N15"/>
+    <hyperlink r:id="rId12" ref="N16"/>
+    <hyperlink r:id="rId13" ref="N17"/>
+    <hyperlink r:id="rId14" ref="N18"/>
+    <hyperlink r:id="rId15" ref="N19"/>
+    <hyperlink r:id="rId16" ref="N20"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <drawing r:id="rId10"/>
-  <legacyDrawing r:id="rId11"/>
+  <drawing r:id="rId17"/>
+  <legacyDrawing r:id="rId18"/>
 </worksheet>
 </file>
</xml_diff>